<commit_message>
code update for dcd
</commit_message>
<xml_diff>
--- a/r-material-examined/data/Platigaster group export 2023-07-05 clavatus only test.xlsx
+++ b/r-material-examined/data/Platigaster group export 2023-07-05 clavatus only test.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10311"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilydarling/Documents/GitHub/r-taxonomy/r-material-examined/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ACB381CE-AE88-47EF-A664-D788A27C1549}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8147C38F-B763-9A43-845E-CC23532DE819}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{80D72645-C7FD-4BA4-9675-72D01261A180}"/>
+    <workbookView xWindow="1200" yWindow="4060" windowWidth="29040" windowHeight="15720" xr2:uid="{80D72645-C7FD-4BA4-9675-72D01261A180}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1464,7 +1464,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2168,9 +2168,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D243A71-0FB0-4AE2-AA3E-DAA82BEB1B2C}">
   <dimension ref="A1:BA38"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="12" max="12" width="19" customWidth="1"/>
+    <col min="26" max="26" width="23" customWidth="1"/>
+    <col min="28" max="28" width="19.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:53" s="20" customFormat="1" ht="99.75" customHeight="1">
+    <row r="1" spans="1:53" s="20" customFormat="1" ht="99.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2327,7 +2332,7 @@
       <c r="AZ1" s="2"/>
       <c r="BA1" s="2"/>
     </row>
-    <row r="2" spans="1:53" s="26" customFormat="1">
+    <row r="2" spans="1:53" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="21">
         <v>3099</v>
       </c>
@@ -2432,7 +2437,7 @@
       <c r="AY2" s="23"/>
       <c r="AZ2" s="23"/>
     </row>
-    <row r="3" spans="1:53" s="26" customFormat="1">
+    <row r="3" spans="1:53" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="21">
         <v>3098</v>
       </c>
@@ -2539,7 +2544,7 @@
       <c r="AY3" s="23"/>
       <c r="AZ3" s="23"/>
     </row>
-    <row r="4" spans="1:53" s="26" customFormat="1">
+    <row r="4" spans="1:53" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="21">
         <v>2991</v>
       </c>
@@ -2636,7 +2641,7 @@
       <c r="AY4" s="23"/>
       <c r="AZ4" s="23"/>
     </row>
-    <row r="5" spans="1:53" s="26" customFormat="1">
+    <row r="5" spans="1:53" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="21">
         <v>2479</v>
       </c>
@@ -2730,7 +2735,7 @@
       <c r="AY5" s="23"/>
       <c r="AZ5" s="23"/>
     </row>
-    <row r="6" spans="1:53" s="26" customFormat="1">
+    <row r="6" spans="1:53" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="35">
         <v>2473</v>
       </c>
@@ -2812,7 +2817,7 @@
         <v>2450</v>
       </c>
     </row>
-    <row r="7" spans="1:53" s="26" customFormat="1">
+    <row r="7" spans="1:53" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" s="35">
         <v>2472</v>
       </c>
@@ -2897,7 +2902,7 @@
       </c>
       <c r="AU7" s="39"/>
     </row>
-    <row r="8" spans="1:53" s="26" customFormat="1">
+    <row r="8" spans="1:53" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" s="21">
         <v>2471</v>
       </c>
@@ -3009,7 +3014,7 @@
       <c r="AY8" s="23"/>
       <c r="AZ8" s="23"/>
     </row>
-    <row r="9" spans="1:53" s="26" customFormat="1">
+    <row r="9" spans="1:53" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9" s="21">
         <v>2470</v>
       </c>
@@ -3107,7 +3112,7 @@
       <c r="AY9" s="23"/>
       <c r="AZ9" s="23"/>
     </row>
-    <row r="10" spans="1:53" s="26" customFormat="1">
+    <row r="10" spans="1:53" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="21">
         <v>2469</v>
       </c>
@@ -3204,7 +3209,7 @@
       <c r="AY10" s="23"/>
       <c r="AZ10" s="23"/>
     </row>
-    <row r="11" spans="1:53" s="26" customFormat="1">
+    <row r="11" spans="1:53" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="35">
         <v>2468</v>
       </c>
@@ -3289,7 +3294,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="12" spans="1:53" s="26" customFormat="1">
+    <row r="12" spans="1:53" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A12" s="35">
         <v>2414</v>
       </c>
@@ -3375,7 +3380,7 @@
       <c r="AU12" s="39"/>
       <c r="AZ12" s="23"/>
     </row>
-    <row r="13" spans="1:53" s="26" customFormat="1">
+    <row r="13" spans="1:53" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A13" s="35">
         <v>1995</v>
       </c>
@@ -3448,7 +3453,7 @@
       </c>
       <c r="AU13" s="39"/>
     </row>
-    <row r="14" spans="1:53" s="26" customFormat="1">
+    <row r="14" spans="1:53" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="21">
         <v>550</v>
       </c>
@@ -3547,7 +3552,7 @@
       <c r="AY14" s="23"/>
       <c r="AZ14" s="23"/>
     </row>
-    <row r="15" spans="1:53" s="26" customFormat="1">
+    <row r="15" spans="1:53" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="21">
         <v>549</v>
       </c>
@@ -3645,7 +3650,7 @@
       <c r="AY15" s="23"/>
       <c r="AZ15" s="23"/>
     </row>
-    <row r="16" spans="1:53" s="26" customFormat="1">
+    <row r="16" spans="1:53" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="21">
         <v>545</v>
       </c>
@@ -3741,7 +3746,7 @@
       <c r="AY16" s="23"/>
       <c r="AZ16" s="23"/>
     </row>
-    <row r="17" spans="1:52" s="26" customFormat="1">
+    <row r="17" spans="1:52" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A17" s="35">
         <v>540</v>
       </c>
@@ -3832,7 +3837,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="18" spans="1:52" s="26" customFormat="1">
+    <row r="18" spans="1:52" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A18" s="35">
         <v>539</v>
       </c>
@@ -3923,7 +3928,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="19" spans="1:52" s="26" customFormat="1">
+    <row r="19" spans="1:52" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A19" s="35">
         <v>538</v>
       </c>
@@ -4012,7 +4017,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="20" spans="1:52" s="26" customFormat="1">
+    <row r="20" spans="1:52" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A20" s="35">
         <v>537</v>
       </c>
@@ -4101,7 +4106,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="21" spans="1:52" s="26" customFormat="1">
+    <row r="21" spans="1:52" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A21" s="21">
         <v>523</v>
       </c>
@@ -4205,7 +4210,7 @@
       <c r="AY21" s="23"/>
       <c r="AZ21" s="23"/>
     </row>
-    <row r="22" spans="1:52" s="26" customFormat="1">
+    <row r="22" spans="1:52" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A22" s="35">
         <v>522</v>
       </c>
@@ -4285,7 +4290,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="23" spans="1:52" s="26" customFormat="1">
+    <row r="23" spans="1:52" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A23" s="35">
         <v>521</v>
       </c>
@@ -4365,7 +4370,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="24" spans="1:52" s="26" customFormat="1">
+    <row r="24" spans="1:52" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A24" s="35">
         <v>519</v>
       </c>
@@ -4448,7 +4453,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="25" spans="1:52" s="26" customFormat="1">
+    <row r="25" spans="1:52" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A25" s="21">
         <v>516</v>
       </c>
@@ -4553,7 +4558,7 @@
       <c r="AY25" s="23"/>
       <c r="AZ25" s="23"/>
     </row>
-    <row r="26" spans="1:52" s="26" customFormat="1">
+    <row r="26" spans="1:52" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A26" s="35">
         <v>515</v>
       </c>
@@ -4649,7 +4654,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="27" spans="1:52" s="26" customFormat="1">
+    <row r="27" spans="1:52" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A27" s="21">
         <v>509</v>
       </c>
@@ -4759,7 +4764,7 @@
       <c r="AY27" s="23"/>
       <c r="AZ27" s="23"/>
     </row>
-    <row r="28" spans="1:52" s="26" customFormat="1">
+    <row r="28" spans="1:52" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A28" s="35">
         <v>508</v>
       </c>
@@ -4855,7 +4860,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="29" spans="1:52" s="26" customFormat="1">
+    <row r="29" spans="1:52" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A29" s="21">
         <v>507</v>
       </c>
@@ -4967,7 +4972,7 @@
       <c r="AY29" s="23"/>
       <c r="AZ29" s="23"/>
     </row>
-    <row r="30" spans="1:52" s="26" customFormat="1">
+    <row r="30" spans="1:52" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A30" s="35">
         <v>506</v>
       </c>
@@ -5063,7 +5068,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="31" spans="1:52" s="26" customFormat="1">
+    <row r="31" spans="1:52" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A31" s="35">
         <v>505</v>
       </c>
@@ -5163,7 +5168,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="32" spans="1:52" s="26" customFormat="1">
+    <row r="32" spans="1:52" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A32" s="35">
         <v>491</v>
       </c>
@@ -5259,7 +5264,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="33" spans="1:53" s="26" customFormat="1">
+    <row r="33" spans="1:53" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A33" s="35">
         <v>489</v>
       </c>
@@ -5359,7 +5364,7 @@
       </c>
       <c r="BA33" s="25"/>
     </row>
-    <row r="34" spans="1:53" s="26" customFormat="1">
+    <row r="34" spans="1:53" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A34" s="35">
         <v>487</v>
       </c>
@@ -5458,7 +5463,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="35" spans="1:53" s="26" customFormat="1">
+    <row r="35" spans="1:53" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A35" s="35">
         <v>486</v>
       </c>
@@ -5557,7 +5562,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="36" spans="1:53" s="25" customFormat="1">
+    <row r="36" spans="1:53" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A36" s="35">
         <v>485</v>
       </c>
@@ -5669,7 +5674,7 @@
       <c r="AZ36" s="26"/>
       <c r="BA36" s="26"/>
     </row>
-    <row r="37" spans="1:53" s="26" customFormat="1">
+    <row r="37" spans="1:53" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A37" s="35">
         <v>459</v>
       </c>
@@ -5766,7 +5771,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="38" spans="1:53" s="26" customFormat="1">
+    <row r="38" spans="1:53" s="26" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A38" s="49"/>
       <c r="O38" s="45"/>
       <c r="P38" s="45"/>

</xml_diff>